<commit_message>
fix(template): numFmt durata Rumore '[hh]:mm:ss' via tools/fix-rumore-template.py
</commit_message>
<xml_diff>
--- a/public/templates/rumore.xlsx
+++ b/public/templates/rumore.xlsx
@@ -18,7 +18,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="[hh]:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="0.0"/>
+  </numFmts>
   <fonts count="4">
     <font>
       <name val="Calibri"/>
@@ -86,7 +89,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -117,6 +120,12 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -583,104 +592,104 @@
       <c r="A4" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="7" t="n"/>
+      <c r="B4" s="11" t="n"/>
       <c r="C4" s="7" t="n"/>
       <c r="D4" s="7" t="n"/>
       <c r="E4" s="7" t="n"/>
-      <c r="F4" s="7" t="n"/>
-      <c r="G4" s="7" t="n"/>
-      <c r="H4" s="7" t="n"/>
+      <c r="F4" s="12" t="n"/>
+      <c r="G4" s="12" t="n"/>
+      <c r="H4" s="12" t="n"/>
       <c r="I4" s="7" t="n"/>
     </row>
     <row r="5" ht="36" customHeight="1">
       <c r="A5" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="7" t="n"/>
+      <c r="B5" s="11" t="n"/>
       <c r="C5" s="7" t="n"/>
       <c r="D5" s="7" t="n"/>
       <c r="E5" s="7" t="n"/>
-      <c r="F5" s="7" t="n"/>
-      <c r="G5" s="7" t="n"/>
-      <c r="H5" s="7" t="n"/>
+      <c r="F5" s="12" t="n"/>
+      <c r="G5" s="12" t="n"/>
+      <c r="H5" s="12" t="n"/>
       <c r="I5" s="7" t="n"/>
     </row>
     <row r="6" ht="36" customHeight="1">
       <c r="A6" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="7" t="n"/>
+      <c r="B6" s="11" t="n"/>
       <c r="C6" s="7" t="n"/>
       <c r="D6" s="7" t="n"/>
       <c r="E6" s="7" t="n"/>
-      <c r="F6" s="7" t="n"/>
-      <c r="G6" s="7" t="n"/>
-      <c r="H6" s="7" t="n"/>
+      <c r="F6" s="12" t="n"/>
+      <c r="G6" s="12" t="n"/>
+      <c r="H6" s="12" t="n"/>
       <c r="I6" s="7" t="n"/>
     </row>
     <row r="7" ht="36" customHeight="1">
       <c r="A7" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="7" t="n"/>
+      <c r="B7" s="11" t="n"/>
       <c r="C7" s="7" t="n"/>
       <c r="D7" s="7" t="n"/>
       <c r="E7" s="7" t="n"/>
-      <c r="F7" s="7" t="n"/>
-      <c r="G7" s="7" t="n"/>
-      <c r="H7" s="7" t="n"/>
+      <c r="F7" s="12" t="n"/>
+      <c r="G7" s="12" t="n"/>
+      <c r="H7" s="12" t="n"/>
       <c r="I7" s="7" t="n"/>
     </row>
     <row r="8" ht="36" customHeight="1">
       <c r="A8" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="7" t="n"/>
+      <c r="B8" s="11" t="n"/>
       <c r="C8" s="7" t="n"/>
       <c r="D8" s="7" t="n"/>
       <c r="E8" s="7" t="n"/>
-      <c r="F8" s="7" t="n"/>
-      <c r="G8" s="7" t="n"/>
-      <c r="H8" s="7" t="n"/>
+      <c r="F8" s="12" t="n"/>
+      <c r="G8" s="12" t="n"/>
+      <c r="H8" s="12" t="n"/>
       <c r="I8" s="7" t="n"/>
     </row>
     <row r="9" ht="36" customHeight="1">
       <c r="A9" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="7" t="n"/>
+      <c r="B9" s="11" t="n"/>
       <c r="C9" s="7" t="n"/>
       <c r="D9" s="7" t="n"/>
       <c r="E9" s="7" t="n"/>
-      <c r="F9" s="7" t="n"/>
-      <c r="G9" s="7" t="n"/>
-      <c r="H9" s="7" t="n"/>
+      <c r="F9" s="12" t="n"/>
+      <c r="G9" s="12" t="n"/>
+      <c r="H9" s="12" t="n"/>
       <c r="I9" s="7" t="n"/>
     </row>
     <row r="10" ht="36" customHeight="1">
       <c r="A10" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="7" t="n"/>
+      <c r="B10" s="11" t="n"/>
       <c r="C10" s="7" t="n"/>
       <c r="D10" s="7" t="n"/>
       <c r="E10" s="7" t="n"/>
-      <c r="F10" s="7" t="n"/>
-      <c r="G10" s="7" t="n"/>
-      <c r="H10" s="7" t="n"/>
+      <c r="F10" s="12" t="n"/>
+      <c r="G10" s="12" t="n"/>
+      <c r="H10" s="12" t="n"/>
       <c r="I10" s="7" t="n"/>
     </row>
     <row r="11" ht="36" customHeight="1">
       <c r="A11" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="7" t="n"/>
+      <c r="B11" s="11" t="n"/>
       <c r="C11" s="7" t="n"/>
       <c r="D11" s="7" t="n"/>
       <c r="E11" s="7" t="n"/>
-      <c r="F11" s="7" t="n"/>
-      <c r="G11" s="7" t="n"/>
-      <c r="H11" s="7" t="n"/>
+      <c r="F11" s="12" t="n"/>
+      <c r="G11" s="12" t="n"/>
+      <c r="H11" s="12" t="n"/>
       <c r="I11" s="7" t="n"/>
     </row>
     <row r="12" ht="15" customHeight="1"/>
@@ -785,104 +794,104 @@
       <c r="A19" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="B19" s="7" t="n"/>
+      <c r="B19" s="11" t="n"/>
       <c r="C19" s="7" t="n"/>
       <c r="D19" s="7" t="n"/>
       <c r="E19" s="7" t="n"/>
-      <c r="F19" s="7" t="n"/>
-      <c r="G19" s="7" t="n"/>
-      <c r="H19" s="7" t="n"/>
+      <c r="F19" s="12" t="n"/>
+      <c r="G19" s="12" t="n"/>
+      <c r="H19" s="12" t="n"/>
       <c r="I19" s="7" t="n"/>
     </row>
     <row r="20" ht="36" customHeight="1">
       <c r="A20" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="B20" s="7" t="n"/>
+      <c r="B20" s="11" t="n"/>
       <c r="C20" s="7" t="n"/>
       <c r="D20" s="7" t="n"/>
       <c r="E20" s="7" t="n"/>
-      <c r="F20" s="7" t="n"/>
-      <c r="G20" s="7" t="n"/>
-      <c r="H20" s="7" t="n"/>
+      <c r="F20" s="12" t="n"/>
+      <c r="G20" s="12" t="n"/>
+      <c r="H20" s="12" t="n"/>
       <c r="I20" s="7" t="n"/>
     </row>
     <row r="21" ht="36" customHeight="1">
       <c r="A21" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="B21" s="7" t="n"/>
+      <c r="B21" s="11" t="n"/>
       <c r="C21" s="7" t="n"/>
       <c r="D21" s="7" t="n"/>
       <c r="E21" s="7" t="n"/>
-      <c r="F21" s="7" t="n"/>
-      <c r="G21" s="7" t="n"/>
-      <c r="H21" s="7" t="n"/>
+      <c r="F21" s="12" t="n"/>
+      <c r="G21" s="12" t="n"/>
+      <c r="H21" s="12" t="n"/>
       <c r="I21" s="7" t="n"/>
     </row>
     <row r="22" ht="36" customHeight="1">
       <c r="A22" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="B22" s="7" t="n"/>
+      <c r="B22" s="11" t="n"/>
       <c r="C22" s="7" t="n"/>
       <c r="D22" s="7" t="n"/>
       <c r="E22" s="7" t="n"/>
-      <c r="F22" s="7" t="n"/>
-      <c r="G22" s="7" t="n"/>
-      <c r="H22" s="7" t="n"/>
+      <c r="F22" s="12" t="n"/>
+      <c r="G22" s="12" t="n"/>
+      <c r="H22" s="12" t="n"/>
       <c r="I22" s="7" t="n"/>
     </row>
     <row r="23" ht="36" customHeight="1">
       <c r="A23" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="B23" s="7" t="n"/>
+      <c r="B23" s="11" t="n"/>
       <c r="C23" s="7" t="n"/>
       <c r="D23" s="7" t="n"/>
       <c r="E23" s="7" t="n"/>
-      <c r="F23" s="7" t="n"/>
-      <c r="G23" s="7" t="n"/>
-      <c r="H23" s="7" t="n"/>
+      <c r="F23" s="12" t="n"/>
+      <c r="G23" s="12" t="n"/>
+      <c r="H23" s="12" t="n"/>
       <c r="I23" s="7" t="n"/>
     </row>
     <row r="24" ht="36" customHeight="1">
       <c r="A24" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="B24" s="7" t="n"/>
+      <c r="B24" s="11" t="n"/>
       <c r="C24" s="7" t="n"/>
       <c r="D24" s="7" t="n"/>
       <c r="E24" s="7" t="n"/>
-      <c r="F24" s="7" t="n"/>
-      <c r="G24" s="7" t="n"/>
-      <c r="H24" s="7" t="n"/>
+      <c r="F24" s="12" t="n"/>
+      <c r="G24" s="12" t="n"/>
+      <c r="H24" s="12" t="n"/>
       <c r="I24" s="7" t="n"/>
     </row>
     <row r="25" ht="36" customHeight="1">
       <c r="A25" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="B25" s="7" t="n"/>
+      <c r="B25" s="11" t="n"/>
       <c r="C25" s="7" t="n"/>
       <c r="D25" s="7" t="n"/>
       <c r="E25" s="7" t="n"/>
-      <c r="F25" s="7" t="n"/>
-      <c r="G25" s="7" t="n"/>
-      <c r="H25" s="7" t="n"/>
+      <c r="F25" s="12" t="n"/>
+      <c r="G25" s="12" t="n"/>
+      <c r="H25" s="12" t="n"/>
       <c r="I25" s="7" t="n"/>
     </row>
     <row r="26" ht="36" customHeight="1">
       <c r="A26" s="6" t="n">
         <v>16</v>
       </c>
-      <c r="B26" s="7" t="n"/>
+      <c r="B26" s="11" t="n"/>
       <c r="C26" s="7" t="n"/>
       <c r="D26" s="7" t="n"/>
       <c r="E26" s="7" t="n"/>
-      <c r="F26" s="7" t="n"/>
-      <c r="G26" s="7" t="n"/>
-      <c r="H26" s="7" t="n"/>
+      <c r="F26" s="12" t="n"/>
+      <c r="G26" s="12" t="n"/>
+      <c r="H26" s="12" t="n"/>
       <c r="I26" s="7" t="n"/>
     </row>
     <row r="27" ht="15" customHeight="1"/>
@@ -987,104 +996,104 @@
       <c r="A34" s="6" t="n">
         <v>17</v>
       </c>
-      <c r="B34" s="7" t="n"/>
+      <c r="B34" s="11" t="n"/>
       <c r="C34" s="7" t="n"/>
       <c r="D34" s="7" t="n"/>
       <c r="E34" s="7" t="n"/>
-      <c r="F34" s="7" t="n"/>
-      <c r="G34" s="7" t="n"/>
-      <c r="H34" s="7" t="n"/>
+      <c r="F34" s="12" t="n"/>
+      <c r="G34" s="12" t="n"/>
+      <c r="H34" s="12" t="n"/>
       <c r="I34" s="7" t="n"/>
     </row>
     <row r="35" ht="36" customHeight="1">
       <c r="A35" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="B35" s="7" t="n"/>
+      <c r="B35" s="11" t="n"/>
       <c r="C35" s="7" t="n"/>
       <c r="D35" s="7" t="n"/>
       <c r="E35" s="7" t="n"/>
-      <c r="F35" s="7" t="n"/>
-      <c r="G35" s="7" t="n"/>
-      <c r="H35" s="7" t="n"/>
+      <c r="F35" s="12" t="n"/>
+      <c r="G35" s="12" t="n"/>
+      <c r="H35" s="12" t="n"/>
       <c r="I35" s="7" t="n"/>
     </row>
     <row r="36" ht="36" customHeight="1">
       <c r="A36" s="6" t="n">
         <v>19</v>
       </c>
-      <c r="B36" s="7" t="n"/>
+      <c r="B36" s="11" t="n"/>
       <c r="C36" s="7" t="n"/>
       <c r="D36" s="7" t="n"/>
       <c r="E36" s="7" t="n"/>
-      <c r="F36" s="7" t="n"/>
-      <c r="G36" s="7" t="n"/>
-      <c r="H36" s="7" t="n"/>
+      <c r="F36" s="12" t="n"/>
+      <c r="G36" s="12" t="n"/>
+      <c r="H36" s="12" t="n"/>
       <c r="I36" s="7" t="n"/>
     </row>
     <row r="37" ht="36" customHeight="1">
       <c r="A37" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="B37" s="7" t="n"/>
+      <c r="B37" s="11" t="n"/>
       <c r="C37" s="7" t="n"/>
       <c r="D37" s="7" t="n"/>
       <c r="E37" s="7" t="n"/>
-      <c r="F37" s="7" t="n"/>
-      <c r="G37" s="7" t="n"/>
-      <c r="H37" s="7" t="n"/>
+      <c r="F37" s="12" t="n"/>
+      <c r="G37" s="12" t="n"/>
+      <c r="H37" s="12" t="n"/>
       <c r="I37" s="7" t="n"/>
     </row>
     <row r="38" ht="36" customHeight="1">
       <c r="A38" s="6" t="n">
         <v>21</v>
       </c>
-      <c r="B38" s="7" t="n"/>
+      <c r="B38" s="11" t="n"/>
       <c r="C38" s="7" t="n"/>
       <c r="D38" s="7" t="n"/>
       <c r="E38" s="7" t="n"/>
-      <c r="F38" s="7" t="n"/>
-      <c r="G38" s="7" t="n"/>
-      <c r="H38" s="7" t="n"/>
+      <c r="F38" s="12" t="n"/>
+      <c r="G38" s="12" t="n"/>
+      <c r="H38" s="12" t="n"/>
       <c r="I38" s="7" t="n"/>
     </row>
     <row r="39" ht="36" customHeight="1">
       <c r="A39" s="6" t="n">
         <v>22</v>
       </c>
-      <c r="B39" s="7" t="n"/>
+      <c r="B39" s="11" t="n"/>
       <c r="C39" s="7" t="n"/>
       <c r="D39" s="7" t="n"/>
       <c r="E39" s="7" t="n"/>
-      <c r="F39" s="7" t="n"/>
-      <c r="G39" s="7" t="n"/>
-      <c r="H39" s="7" t="n"/>
+      <c r="F39" s="12" t="n"/>
+      <c r="G39" s="12" t="n"/>
+      <c r="H39" s="12" t="n"/>
       <c r="I39" s="7" t="n"/>
     </row>
     <row r="40" ht="36" customHeight="1">
       <c r="A40" s="6" t="n">
         <v>23</v>
       </c>
-      <c r="B40" s="7" t="n"/>
+      <c r="B40" s="11" t="n"/>
       <c r="C40" s="7" t="n"/>
       <c r="D40" s="7" t="n"/>
       <c r="E40" s="7" t="n"/>
-      <c r="F40" s="7" t="n"/>
-      <c r="G40" s="7" t="n"/>
-      <c r="H40" s="7" t="n"/>
+      <c r="F40" s="12" t="n"/>
+      <c r="G40" s="12" t="n"/>
+      <c r="H40" s="12" t="n"/>
       <c r="I40" s="7" t="n"/>
     </row>
     <row r="41" ht="36" customHeight="1">
       <c r="A41" s="6" t="n">
         <v>24</v>
       </c>
-      <c r="B41" s="7" t="n"/>
+      <c r="B41" s="11" t="n"/>
       <c r="C41" s="7" t="n"/>
       <c r="D41" s="7" t="n"/>
       <c r="E41" s="7" t="n"/>
-      <c r="F41" s="7" t="n"/>
-      <c r="G41" s="7" t="n"/>
-      <c r="H41" s="7" t="n"/>
+      <c r="F41" s="12" t="n"/>
+      <c r="G41" s="12" t="n"/>
+      <c r="H41" s="12" t="n"/>
       <c r="I41" s="7" t="n"/>
     </row>
     <row r="42" ht="15" customHeight="1"/>
@@ -1189,104 +1198,104 @@
       <c r="A49" s="6" t="n">
         <v>25</v>
       </c>
-      <c r="B49" s="7" t="n"/>
+      <c r="B49" s="11" t="n"/>
       <c r="C49" s="7" t="n"/>
       <c r="D49" s="7" t="n"/>
       <c r="E49" s="7" t="n"/>
-      <c r="F49" s="7" t="n"/>
-      <c r="G49" s="7" t="n"/>
-      <c r="H49" s="7" t="n"/>
+      <c r="F49" s="12" t="n"/>
+      <c r="G49" s="12" t="n"/>
+      <c r="H49" s="12" t="n"/>
       <c r="I49" s="7" t="n"/>
     </row>
     <row r="50" ht="36" customHeight="1">
       <c r="A50" s="6" t="n">
         <v>26</v>
       </c>
-      <c r="B50" s="7" t="n"/>
+      <c r="B50" s="11" t="n"/>
       <c r="C50" s="7" t="n"/>
       <c r="D50" s="7" t="n"/>
       <c r="E50" s="7" t="n"/>
-      <c r="F50" s="7" t="n"/>
-      <c r="G50" s="7" t="n"/>
-      <c r="H50" s="7" t="n"/>
+      <c r="F50" s="12" t="n"/>
+      <c r="G50" s="12" t="n"/>
+      <c r="H50" s="12" t="n"/>
       <c r="I50" s="7" t="n"/>
     </row>
     <row r="51" ht="36" customHeight="1">
       <c r="A51" s="6" t="n">
         <v>27</v>
       </c>
-      <c r="B51" s="7" t="n"/>
+      <c r="B51" s="11" t="n"/>
       <c r="C51" s="7" t="n"/>
       <c r="D51" s="7" t="n"/>
       <c r="E51" s="7" t="n"/>
-      <c r="F51" s="7" t="n"/>
-      <c r="G51" s="7" t="n"/>
-      <c r="H51" s="7" t="n"/>
+      <c r="F51" s="12" t="n"/>
+      <c r="G51" s="12" t="n"/>
+      <c r="H51" s="12" t="n"/>
       <c r="I51" s="7" t="n"/>
     </row>
     <row r="52" ht="36" customHeight="1">
       <c r="A52" s="6" t="n">
         <v>28</v>
       </c>
-      <c r="B52" s="7" t="n"/>
+      <c r="B52" s="11" t="n"/>
       <c r="C52" s="7" t="n"/>
       <c r="D52" s="7" t="n"/>
       <c r="E52" s="7" t="n"/>
-      <c r="F52" s="7" t="n"/>
-      <c r="G52" s="7" t="n"/>
-      <c r="H52" s="7" t="n"/>
+      <c r="F52" s="12" t="n"/>
+      <c r="G52" s="12" t="n"/>
+      <c r="H52" s="12" t="n"/>
       <c r="I52" s="7" t="n"/>
     </row>
     <row r="53" ht="36" customHeight="1">
       <c r="A53" s="6" t="n">
         <v>29</v>
       </c>
-      <c r="B53" s="7" t="n"/>
+      <c r="B53" s="11" t="n"/>
       <c r="C53" s="7" t="n"/>
       <c r="D53" s="7" t="n"/>
       <c r="E53" s="7" t="n"/>
-      <c r="F53" s="7" t="n"/>
-      <c r="G53" s="7" t="n"/>
-      <c r="H53" s="7" t="n"/>
+      <c r="F53" s="12" t="n"/>
+      <c r="G53" s="12" t="n"/>
+      <c r="H53" s="12" t="n"/>
       <c r="I53" s="7" t="n"/>
     </row>
     <row r="54" ht="36" customHeight="1">
       <c r="A54" s="6" t="n">
         <v>30</v>
       </c>
-      <c r="B54" s="7" t="n"/>
+      <c r="B54" s="11" t="n"/>
       <c r="C54" s="7" t="n"/>
       <c r="D54" s="7" t="n"/>
       <c r="E54" s="7" t="n"/>
-      <c r="F54" s="7" t="n"/>
-      <c r="G54" s="7" t="n"/>
-      <c r="H54" s="7" t="n"/>
+      <c r="F54" s="12" t="n"/>
+      <c r="G54" s="12" t="n"/>
+      <c r="H54" s="12" t="n"/>
       <c r="I54" s="7" t="n"/>
     </row>
     <row r="55" ht="36" customHeight="1">
       <c r="A55" s="6" t="n">
         <v>31</v>
       </c>
-      <c r="B55" s="7" t="n"/>
+      <c r="B55" s="11" t="n"/>
       <c r="C55" s="7" t="n"/>
       <c r="D55" s="7" t="n"/>
       <c r="E55" s="7" t="n"/>
-      <c r="F55" s="7" t="n"/>
-      <c r="G55" s="7" t="n"/>
-      <c r="H55" s="7" t="n"/>
+      <c r="F55" s="12" t="n"/>
+      <c r="G55" s="12" t="n"/>
+      <c r="H55" s="12" t="n"/>
       <c r="I55" s="7" t="n"/>
     </row>
     <row r="56" ht="36" customHeight="1">
       <c r="A56" s="6" t="n">
         <v>32</v>
       </c>
-      <c r="B56" s="7" t="n"/>
+      <c r="B56" s="11" t="n"/>
       <c r="C56" s="7" t="n"/>
       <c r="D56" s="7" t="n"/>
       <c r="E56" s="7" t="n"/>
-      <c r="F56" s="7" t="n"/>
-      <c r="G56" s="7" t="n"/>
-      <c r="H56" s="7" t="n"/>
+      <c r="F56" s="12" t="n"/>
+      <c r="G56" s="12" t="n"/>
+      <c r="H56" s="12" t="n"/>
       <c r="I56" s="7" t="n"/>
     </row>
     <row r="57" ht="15" customHeight="1"/>

</xml_diff>